<commit_message>
Prueba Actualizacion de Precios
</commit_message>
<xml_diff>
--- a/catalog/products.xlsx
+++ b/catalog/products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\catalogo_head\Catalogo_Head\catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEFD56AB-346C-4BE5-9C9E-9A9F296A6583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{065960D2-A5AF-42B4-B838-F070B2AFB644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categorias" sheetId="1" r:id="rId1"/>
@@ -9811,7 +9811,7 @@
         <v>150845</v>
       </c>
       <c r="H12" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>142</v>
@@ -9852,7 +9852,7 @@
         <v>123</v>
       </c>
       <c r="G13" s="10">
-        <v>150845</v>
+        <v>200000</v>
       </c>
       <c r="H13" s="6" t="b">
         <v>1</v>
@@ -10346,7 +10346,7 @@
         <v>13</v>
       </c>
       <c r="G24" s="25">
-        <v>18288</v>
+        <v>15000</v>
       </c>
       <c r="H24" s="24" t="b">
         <v>1</v>
@@ -40496,7 +40496,7 @@
         <v>835</v>
       </c>
       <c r="D3" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="7">
         <v>1</v>
@@ -48856,7 +48856,7 @@
         <v>842</v>
       </c>
       <c r="D223" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E223" s="7">
         <v>1</v>

</xml_diff>

<commit_message>
Prueba de Precios/Stock Finalizada
</commit_message>
<xml_diff>
--- a/catalog/products.xlsx
+++ b/catalog/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\catalogo_head\Catalogo_Head\catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{065960D2-A5AF-42B4-B838-F070B2AFB644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{21CB7DC1-3162-40B6-AE2F-C21FC58F6E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9852,7 +9852,7 @@
         <v>123</v>
       </c>
       <c r="G13" s="10">
-        <v>200000</v>
+        <v>150845</v>
       </c>
       <c r="H13" s="6" t="b">
         <v>1</v>
@@ -10346,7 +10346,7 @@
         <v>13</v>
       </c>
       <c r="G24" s="25">
-        <v>15000</v>
+        <v>18288</v>
       </c>
       <c r="H24" s="24" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Prueba de Cambio de Excel en otra PC
</commit_message>
<xml_diff>
--- a/catalog/products.xlsx
+++ b/catalog/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\catalogo_head\Catalogo_Head\catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8E90E8-8FDA-4FC5-823C-D394C4CA52CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E886DF58-055E-4432-BA8E-7B51AFD29277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9855,7 +9855,7 @@
         <v>65</v>
       </c>
       <c r="G12" s="13">
-        <v>150845</v>
+        <v>300000</v>
       </c>
       <c r="H12" s="8" t="b">
         <v>1</v>
@@ -42785,7 +42785,7 @@
         <v>503</v>
       </c>
       <c r="D62" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E62" s="5">
         <v>0</v>
@@ -43431,7 +43431,7 @@
         <v>505</v>
       </c>
       <c r="D79" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E79" s="9">
         <v>1</v>

</xml_diff>